<commit_message>
data: country profile monthly 2026-10-21
</commit_message>
<xml_diff>
--- a/output/country_profile.xlsx
+++ b/output/country_profile.xlsx
@@ -541,12 +541,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.9% (2026.09)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.6% (2026.09)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -603,12 +603,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.9% (2026.09)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.2% (2026.09)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.7% (2026.09)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.2% (2026.09)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -724,12 +724,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.1% (2026.09)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.5% (2026.09)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -781,12 +781,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.3% (2026.09)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.4% (2026.09)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.6% (2026.09)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.8% (2026.08)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -898,12 +898,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.1% (2026.08)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.7% (2026.08)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.1% (2026.09)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.3% (2026 Q2)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1012,12 +1012,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.2% (2026.09)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.2% (2026.08)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.9% (2026.09)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.9% (2026 Q2)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.4% (2026.09)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.0% (2026.09)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1183,12 +1183,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.1% (2026.09)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.8% (2026.08)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1240,12 +1240,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.1% (2026.09)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.1% (2026.09)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1297,12 +1297,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.3% (2026.09)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.2% (2026.08)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1354,12 +1354,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29.7% (2026.09)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.8% (2026.08)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.5% (2026.09)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.0% (2026.09)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10.0% (2026.09)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1525,12 +1525,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.6% (2026.09)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.1% (2026.09)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.1% (2026.09)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.2% (2026 Q2)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1639,12 +1639,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.6% (2026.09)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.4% (2026.08)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1696,12 +1696,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.3% (2026.08)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.5% (2026 Q2)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.7% (2026.09)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.4% (2026.08)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1810,12 +1810,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.5% (2026.09)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.0% (2026.08)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1867,12 +1867,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.3% (2026.09)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.4% (2026.08)</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -1924,12 +1924,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.1% (2026.09)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.6% (2026.08)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1981,12 +1981,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.6% (2026.09)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.3% (2026.08)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.8% (2026.08)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2095,12 +2095,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.3% (2026.09)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.7% (2026 Q1)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.9% (2026.08)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.5% (2026.08)</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2210,12 +2210,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.0% (2026.08)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.7% (2026.09)</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2267,12 +2267,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.8% (2026.09)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.9% (2026.08)</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2324,12 +2324,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.8% (2026.09)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0% (2026 Q1)</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2381,12 +2381,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.1% (2026.09)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.2% (2026 Q2)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2438,12 +2438,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.7% (2026.09)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.3% (2026.08)</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2495,12 +2495,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.3% (2026.08)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.9% (2026 Q2)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.0% (2025.11)</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2609,12 +2609,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13.9% (2026.09)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.8% (2026 Q2)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2666,12 +2666,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.9% (2026.09)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.0% (2026 Q2)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2723,12 +2723,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.3% (2026.09)</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.5% (2026 Q2)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2753,7 +2753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G105"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2834,22 +2834,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>KOR</t>
+          <t>CHN</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>중국</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2863,22 +2863,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>KOR</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>캐나다</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2892,12 +2892,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CHN</t>
+          <t>GBR</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>중국</t>
+          <t>영국</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 값 없음; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2921,80 +2921,88 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CHN</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>중국</t>
+          <t>이탈리아</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
+          <t>법정 최저임금 없음 (단체협약으로 결정)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>각국 노동법 기준</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CHN</t>
+          <t>SWE</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>중국</t>
+          <t>스웨덴</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
+          <t>법정 최저임금 없음 (단체협약으로 결정)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>각국 노동법 기준</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>RUS</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>미국</t>
+          <t>러시아</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -3008,12 +3016,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UKR</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>미국</t>
+          <t>우크라이나</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -3023,7 +3031,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (파싱 실패: 최신 값의 기준 기간을 찾지 못함)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -3031,18 +3039,26 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Trading Economics</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://ko.tradingeconomics.com/ukraine/unemployment-rate</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>AUT</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>캐나다</t>
+          <t>오스트리아</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3052,36 +3068,40 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
+          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>법정 최저임금 없음 (단체협약으로 결정)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>각국 노동법 기준</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>캐나다</t>
+          <t>모로코</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3095,22 +3115,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>캐나다</t>
+          <t>멕시코</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3124,22 +3144,22 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>DEU</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>독일</t>
+          <t>콜롬비아</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -3153,22 +3173,22 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>DEU</t>
+          <t>CHL</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>독일</t>
+          <t>칠레</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3182,22 +3202,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HUN</t>
+          <t>BRA</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>헝가리</t>
+          <t>브라질</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -3211,22 +3231,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HUN</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>헝가리</t>
+          <t>파나마</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -3240,22 +3260,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GBR</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>영국</t>
+          <t>파나마</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>최저임금</t>
+          <t>실업률</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 값 없음; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
+          <t>미갱신 (파싱 실패: 최신 값의 기준 기간을 찾지 못함)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -3263,28 +3283,36 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Trading Economics</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://ko.tradingeconomics.com/panama/unemployment-rate</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GBR</t>
+          <t>IDN</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>영국</t>
+          <t>인도네시아</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -3298,22 +3326,22 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GBR</t>
+          <t>JPN</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>영국</t>
+          <t>일본</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -3327,22 +3355,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>프랑스</t>
+          <t>호주</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -3356,22 +3384,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>MYS</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>프랑스</t>
+          <t>말레이시아</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -3385,12 +3413,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>THA</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>이탈리아</t>
+          <t>태국</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3400,40 +3428,36 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>법정 최저임금 없음 (단체협약으로 결정)</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>각국 노동법 기준</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>이탈리아</t>
+          <t>베트남</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -3447,22 +3471,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>TWN</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>이탈리아</t>
+          <t>대만</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3476,80 +3500,88 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ESP</t>
+          <t>SGP</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>스페인</t>
+          <t>싱가포르</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>법정 최저임금 없음 (업종별 점진임금모델(PWM) 적용)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>각국 노동법 기준</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ESP</t>
+          <t>ARE</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>스페인</t>
+          <t>아랍에미리트</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>법정 최저임금 없음 (자국민 대상 기준만 있음)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>각국 노동법 기준</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>NLD</t>
+          <t>ARE</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>네덜란드</t>
+          <t>아랍에미리트</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>실업률</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (파싱 실패: 최신 값의 기준 기간을 찾지 못함)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -3557,28 +3589,36 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Trading Economics</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>https://ko.tradingeconomics.com/united-arab-emirates/unemployment-rate</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>NLD</t>
+          <t>EGY</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>네덜란드</t>
+          <t>이집트</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3592,51 +3632,55 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>POL</t>
+          <t>SAU</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>폴란드</t>
+          <t>사우디아라비아</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>인플레이션</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
+          <t>법정 최저임금 없음 (자국민 대상 기준만 있음)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>각국 노동법 기준</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>POL</t>
+          <t>KAZ</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>폴란드</t>
+          <t>카자흐스탄</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>실업률</t>
+          <t>최저임금</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3646,2201 +3690,6 @@
       </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>SWE</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>스웨덴</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 (단체협약으로 결정)</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>각국 노동법 기준</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>SWE</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>스웨덴</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>SWE</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>스웨덴</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>RUS</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>러시아</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>RUS</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>러시아</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>RUS</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>러시아</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>TUR</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>튀르키예</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>TUR</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>튀르키예</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>CZE</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>체코</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>CZE</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>체코</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>UKR</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>우크라이나</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>UKR</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>우크라이나</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>AUT</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>오스트리아</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 (단체협약으로 결정)</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>각국 노동법 기준</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>AUT</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>오스트리아</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>AUT</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>오스트리아</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>SRB</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>세르비아</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>SRB</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>세르비아</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>ROU</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>루마니아</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>ROU</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>루마니아</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>모로코</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>모로코</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>모로코</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>HRV</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>크로아티아</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>HRV</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>크로아티아</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>MEX</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>멕시코</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>MEX</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>멕시코</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>MEX</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>멕시코</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>COL</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>콜롬비아</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>COL</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>콜롬비아</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>COL</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>콜롬비아</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>CHL</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>칠레</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>CHL</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>칠레</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>CHL</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>칠레</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>BRA</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>브라질</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>BRA</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>브라질</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>BRA</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>브라질</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>파나마</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>파나마</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>파나마</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>IDN</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>인도네시아</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>IDN</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>인도네시아</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>IDN</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>인도네시아</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>JPN</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>일본</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>JPN</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>일본</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>JPN</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>일본</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>AUS</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>AUS</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>AUS</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>MYS</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>말레이시아</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>MYS</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>말레이시아</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>MYS</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>말레이시아</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>THA</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>태국</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="2" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>THA</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>태국</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" s="2" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>THA</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>태국</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="2" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>VNM</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>베트남</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="2" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>VNM</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>베트남</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>VNM</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>베트남</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" s="2" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>TWN</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>대만</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>TWN</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>대만</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="2" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>TWN</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>대만</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>SGP</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 (업종별 점진임금모델(PWM) 적용)</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>각국 노동법 기준</t>
-        </is>
-      </c>
-      <c r="G91" s="2" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>SGP</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>SGP</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="2" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>ARE</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>아랍에미리트</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 (자국민 대상 기준만 있음)</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>각국 노동법 기준</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>ARE</t>
-        </is>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>아랍에미리트</t>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="2" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>ARE</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>아랍에미리트</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="2" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>EGY</t>
-        </is>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>이집트</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="2" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>EGY</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>이집트</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="2" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>EGY</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>이집트</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="2" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>SAU</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>사우디아라비아</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 / 검토 필요: 보정 파일 확인일 비어 있음</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>법정 최저임금 없음 (자국민 대상 기준만 있음)</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>각국 노동법 기준</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>SAU</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>사우디아라비아</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="inlineStr"/>
-      <c r="G101" s="2" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>SAU</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>사우디아라비아</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="inlineStr"/>
-      <c r="G102" s="2" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>KAZ</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="inlineStr">
-        <is>
-          <t>카자흐스탄</t>
-        </is>
-      </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>최저임금</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>미갱신 (보정 파일 없음; Eurostat 대상 아님; ILOSTAT 요청 실패: HTTP 400; 직전 값 없음)</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr"/>
-      <c r="G103" s="2" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>KAZ</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>카자흐스탄</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>인플레이션</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" s="2" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>KAZ</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>카자흐스탄</t>
-        </is>
-      </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>실업률</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr"/>
-      <c r="G105" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5864,7 +3713,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-20T16:48:44+09:00</t>
+          <t>2026-10-21T08:10:58+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>